<commit_message>
Updated EPU until 2025
</commit_message>
<xml_diff>
--- a/T20-Brief/G20.xlsx
+++ b/T20-Brief/G20.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e46a4301436fbcaf/Kalyan/KK-Python/Kalyan-Jupyter-Notebooks/T20-Brief/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="107" documentId="8_{ECA320E5-6C1F-3347-AD78-8ED33AE7301E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{975FC2C4-BDD5-C448-8E1F-53D98C3E565E}"/>
+  <xr:revisionPtr revIDLastSave="112" documentId="8_{ECA320E5-6C1F-3347-AD78-8ED33AE7301E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D4D51CC-FA1A-CD41-AC24-FD5A3B3D9E38}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="1000" windowWidth="27640" windowHeight="15100" activeTab="4" xr2:uid="{609D964B-ECF1-144B-A45E-3CDC5CDDA627}"/>
+    <workbookView xWindow="10420" yWindow="780" windowWidth="27640" windowHeight="15100" xr2:uid="{609D964B-ECF1-144B-A45E-3CDC5CDDA627}"/>
   </bookViews>
   <sheets>
     <sheet name="G20-EPU" sheetId="2" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="82">
   <si>
     <t>Year</t>
   </si>
@@ -526,6 +526,15 @@
   <si>
     <t>Country</t>
   </si>
+  <si>
+    <t>2023</t>
+  </si>
+  <si>
+    <t>2024</t>
+  </si>
+  <si>
+    <t>2025</t>
+  </si>
 </sst>
 </file>
 
@@ -646,7 +655,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFill="1"/>
@@ -674,6 +683,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4783,7 +4793,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B40E1B25-B83E-E742-8CDB-C7ECF472B3AB}">
-  <dimension ref="A1:R313"/>
+  <dimension ref="A1:R346"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.1640625" bestFit="1" customWidth="1"/>
@@ -8920,7 +8930,7 @@
         <v>84.128320000000002</v>
       </c>
       <c r="I74" s="11">
-        <v>49.281799999999997</v>
+        <v>49.281837463378906</v>
       </c>
       <c r="J74" s="11">
         <v>126</v>
@@ -8976,7 +8986,7 @@
         <v>230.90960000000001</v>
       </c>
       <c r="I75" s="11">
-        <v>69.260099999999994</v>
+        <v>69.260139465332031</v>
       </c>
       <c r="J75" s="11">
         <v>126</v>
@@ -9032,7 +9042,7 @@
         <v>230.06299999999999</v>
       </c>
       <c r="I76" s="11">
-        <v>113.419</v>
+        <v>113.4190673828125</v>
       </c>
       <c r="J76" s="11">
         <v>143</v>
@@ -9088,7 +9098,7 @@
         <v>155.8158</v>
       </c>
       <c r="I77" s="11">
-        <v>80.293400000000005</v>
+        <v>80.293449401855469</v>
       </c>
       <c r="J77" s="11">
         <v>110</v>
@@ -9144,7 +9154,7 @@
         <v>120.4397</v>
       </c>
       <c r="I78" s="11">
-        <v>62.9846</v>
+        <v>62.984580993652344</v>
       </c>
       <c r="J78" s="11">
         <v>150</v>
@@ -9200,7 +9210,7 @@
         <v>78.666079999999994</v>
       </c>
       <c r="I79" s="11">
-        <v>57.718200000000003</v>
+        <v>57.718231201171875</v>
       </c>
       <c r="J79" s="11">
         <v>82.6</v>
@@ -9256,7 +9266,7 @@
         <v>59.33775</v>
       </c>
       <c r="I80" s="11">
-        <v>63.987699999999997</v>
+        <v>63.987739562988281</v>
       </c>
       <c r="J80" s="11">
         <v>95</v>
@@ -9312,7 +9322,7 @@
         <v>59.89029</v>
       </c>
       <c r="I81" s="11">
-        <v>59.849200000000003</v>
+        <v>59.849166870117188</v>
       </c>
       <c r="J81" s="11">
         <v>79.400000000000006</v>
@@ -9368,7 +9378,7 @@
         <v>89.456360000000004</v>
       </c>
       <c r="I82" s="11">
-        <v>53.425199999999997</v>
+        <v>53.425193786621094</v>
       </c>
       <c r="J82" s="11">
         <v>88.5</v>
@@ -9424,7 +9434,7 @@
         <v>87.1267</v>
       </c>
       <c r="I83" s="11">
-        <v>64.714600000000004</v>
+        <v>64.714637756347656</v>
       </c>
       <c r="J83" s="11">
         <v>103</v>
@@ -9480,7 +9490,7 @@
         <v>106.2878</v>
       </c>
       <c r="I84" s="11">
-        <v>40.537100000000002</v>
+        <v>40.537143707275391</v>
       </c>
       <c r="J84" s="11">
         <v>82.6</v>
@@ -9536,7 +9546,7 @@
         <v>61.571719999999999</v>
       </c>
       <c r="I85" s="11">
-        <v>42.959200000000003</v>
+        <v>42.959209442138672</v>
       </c>
       <c r="J85" s="11">
         <v>94.5</v>
@@ -9592,7 +9602,7 @@
         <v>59.477989999999998</v>
       </c>
       <c r="I86" s="11">
-        <v>77.310500000000005</v>
+        <v>77.310493469238281</v>
       </c>
       <c r="J86" s="11">
         <v>92.2</v>
@@ -9648,7 +9658,7 @@
         <v>83.925870000000003</v>
       </c>
       <c r="I87" s="11">
-        <v>82.817800000000005</v>
+        <v>82.817840576171875</v>
       </c>
       <c r="J87" s="11">
         <v>73.7</v>
@@ -9704,7 +9714,7 @@
         <v>117.33880000000001</v>
       </c>
       <c r="I88" s="11">
-        <v>24.939800000000002</v>
+        <v>24.939825057983398</v>
       </c>
       <c r="J88" s="11">
         <v>135</v>
@@ -9760,7 +9770,7 @@
         <v>104.8796</v>
       </c>
       <c r="I89" s="11">
-        <v>73.950400000000002</v>
+        <v>73.950408935546875</v>
       </c>
       <c r="J89" s="11">
         <v>107</v>
@@ -9816,7 +9826,7 @@
         <v>126.78749999999999</v>
       </c>
       <c r="I90" s="11">
-        <v>229.63300000000001</v>
+        <v>229.63282775878906</v>
       </c>
       <c r="J90" s="11">
         <v>91.1</v>
@@ -9872,7 +9882,7 @@
         <v>104.789</v>
       </c>
       <c r="I91" s="11">
-        <v>48.421300000000002</v>
+        <v>48.421302795410156</v>
       </c>
       <c r="J91" s="11">
         <v>104</v>
@@ -9928,7 +9938,7 @@
         <v>57.157730000000001</v>
       </c>
       <c r="I92" s="11">
-        <v>47.164499999999997</v>
+        <v>47.164531707763672</v>
       </c>
       <c r="J92" s="11">
         <v>168</v>
@@ -9984,7 +9994,7 @@
         <v>60.641840000000002</v>
       </c>
       <c r="I93" s="11">
-        <v>83.190600000000003</v>
+        <v>83.190597534179688</v>
       </c>
       <c r="J93" s="11">
         <v>77</v>
@@ -10040,7 +10050,7 @@
         <v>65.458060000000003</v>
       </c>
       <c r="I94" s="11">
-        <v>41.460900000000002</v>
+        <v>41.460868835449219</v>
       </c>
       <c r="J94" s="11">
         <v>92.8</v>
@@ -10096,7 +10106,7 @@
         <v>115.98439999999999</v>
       </c>
       <c r="I95" s="11">
-        <v>86.207800000000006</v>
+        <v>86.207786560058594</v>
       </c>
       <c r="J95" s="11">
         <v>96.1</v>
@@ -10152,7 +10162,7 @@
         <v>68.121669999999995</v>
       </c>
       <c r="I96" s="11">
-        <v>50.963700000000003</v>
+        <v>50.963676452636719</v>
       </c>
       <c r="J96" s="11">
         <v>133</v>
@@ -10208,7 +10218,7 @@
         <v>54.962209999999999</v>
       </c>
       <c r="I97" s="11">
-        <v>50.826500000000003</v>
+        <v>50.826522827148438</v>
       </c>
       <c r="J97" s="11">
         <v>103</v>
@@ -10264,7 +10274,7 @@
         <v>48.379840000000002</v>
       </c>
       <c r="I98" s="11">
-        <v>52.3063</v>
+        <v>52.306331634521484</v>
       </c>
       <c r="J98" s="11">
         <v>65</v>
@@ -10320,7 +10330,7 @@
         <v>53.162430000000001</v>
       </c>
       <c r="I99" s="11">
-        <v>60.799300000000002</v>
+        <v>60.799285888671875</v>
       </c>
       <c r="J99" s="11">
         <v>89.4</v>
@@ -10376,7 +10386,7 @@
         <v>40.669960000000003</v>
       </c>
       <c r="I100" s="11">
-        <v>38.825299999999999</v>
+        <v>38.825347900390625</v>
       </c>
       <c r="J100" s="11">
         <v>103</v>
@@ -10432,7 +10442,7 @@
         <v>34.60284</v>
       </c>
       <c r="I101" s="11">
-        <v>90.298299999999998</v>
+        <v>90.298301696777344</v>
       </c>
       <c r="J101" s="11">
         <v>104</v>
@@ -10488,7 +10498,7 @@
         <v>66.399050000000003</v>
       </c>
       <c r="I102" s="11">
-        <v>60.122100000000003</v>
+        <v>60.122066497802734</v>
       </c>
       <c r="J102" s="11">
         <v>104</v>
@@ -10544,7 +10554,7 @@
         <v>95.044060000000002</v>
       </c>
       <c r="I103" s="11">
-        <v>63.020299999999999</v>
+        <v>63.020267486572266</v>
       </c>
       <c r="J103" s="11">
         <v>87.7</v>
@@ -10600,7 +10610,7 @@
         <v>80.359679999999997</v>
       </c>
       <c r="I104" s="11">
-        <v>66.427000000000007</v>
+        <v>66.427009582519531</v>
       </c>
       <c r="J104" s="11">
         <v>81.5</v>
@@ -10656,7 +10666,7 @@
         <v>68.518010000000004</v>
       </c>
       <c r="I105" s="11">
-        <v>30.6938</v>
+        <v>30.693752288818359</v>
       </c>
       <c r="J105" s="11">
         <v>90.1</v>
@@ -10712,7 +10722,7 @@
         <v>202.5643</v>
       </c>
       <c r="I106" s="11">
-        <v>31.904399999999999</v>
+        <v>31.904401779174805</v>
       </c>
       <c r="J106" s="11">
         <v>136</v>
@@ -10768,7 +10778,7 @@
         <v>83.171999999999997</v>
       </c>
       <c r="I107" s="11">
-        <v>51.6389</v>
+        <v>51.638874053955078</v>
       </c>
       <c r="J107" s="11">
         <v>55.5</v>
@@ -10824,7 +10834,7 @@
         <v>140.06549999999999</v>
       </c>
       <c r="I108" s="11">
-        <v>33.007199999999997</v>
+        <v>33.007221221923828</v>
       </c>
       <c r="J108" s="11">
         <v>74.5</v>
@@ -10880,7 +10890,7 @@
         <v>63.615409999999997</v>
       </c>
       <c r="I109" s="11">
-        <v>42.346499999999999</v>
+        <v>42.346542358398438</v>
       </c>
       <c r="J109" s="11">
         <v>71.599999999999994</v>
@@ -10936,7 +10946,7 @@
         <v>88.123400000000004</v>
       </c>
       <c r="I110" s="11">
-        <v>39.990200000000002</v>
+        <v>39.990150451660156</v>
       </c>
       <c r="J110" s="11">
         <v>95</v>
@@ -10992,7 +11002,7 @@
         <v>76.186719999999994</v>
       </c>
       <c r="I111" s="11">
-        <v>31.3734</v>
+        <v>31.373428344726562</v>
       </c>
       <c r="J111" s="11">
         <v>43.3</v>
@@ -11048,7 +11058,7 @@
         <v>94.212900000000005</v>
       </c>
       <c r="I112" s="11">
-        <v>32.2682</v>
+        <v>32.268180847167969</v>
       </c>
       <c r="J112" s="11">
         <v>73.5</v>
@@ -11104,7 +11114,7 @@
         <v>79.127499999999998</v>
       </c>
       <c r="I113" s="11">
-        <v>37.325099999999999</v>
+        <v>37.325069427490234</v>
       </c>
       <c r="J113" s="11">
         <v>114</v>
@@ -11160,7 +11170,7 @@
         <v>71.288550000000001</v>
       </c>
       <c r="I114" s="11">
-        <v>39.594000000000001</v>
+        <v>39.594005584716797</v>
       </c>
       <c r="J114" s="11">
         <v>58.4</v>
@@ -11216,7 +11226,7 @@
         <v>105.8366</v>
       </c>
       <c r="I115" s="11">
-        <v>53.543900000000001</v>
+        <v>53.543903350830078</v>
       </c>
       <c r="J115" s="11">
         <v>61.9</v>
@@ -11272,7 +11282,7 @@
         <v>98.154169999999993</v>
       </c>
       <c r="I116" s="11">
-        <v>72.427899999999994</v>
+        <v>72.427879333496094</v>
       </c>
       <c r="J116" s="11">
         <v>64.3</v>
@@ -11328,7 +11338,7 @@
         <v>59.319839999999999</v>
       </c>
       <c r="I117" s="11">
-        <v>59.809899999999999</v>
+        <v>59.809848785400391</v>
       </c>
       <c r="J117" s="11">
         <v>52.2</v>
@@ -11384,7 +11394,7 @@
         <v>93.781329999999997</v>
       </c>
       <c r="I118" s="11">
-        <v>41.711799999999997</v>
+        <v>41.711822509765625</v>
       </c>
       <c r="J118" s="11">
         <v>67.099999999999994</v>
@@ -11440,7 +11450,7 @@
         <v>54.061630000000001</v>
       </c>
       <c r="I119" s="11">
-        <v>37.2012</v>
+        <v>37.201198577880859</v>
       </c>
       <c r="J119" s="11">
         <v>64.099999999999994</v>
@@ -11496,7 +11506,7 @@
         <v>71.951939999999993</v>
       </c>
       <c r="I120" s="11">
-        <v>85.049899999999994</v>
+        <v>85.049903869628906</v>
       </c>
       <c r="J120" s="11">
         <v>71</v>
@@ -11552,7 +11562,7 @@
         <v>84.137990000000002</v>
       </c>
       <c r="I121" s="11">
-        <v>63.4955</v>
+        <v>63.495506286621094</v>
       </c>
       <c r="J121" s="11">
         <v>67.5</v>
@@ -11608,7 +11618,7 @@
         <v>74.495670000000004</v>
       </c>
       <c r="I122" s="11">
-        <v>45.917900000000003</v>
+        <v>45.917915344238281</v>
       </c>
       <c r="J122" s="11">
         <v>32</v>
@@ -11664,7 +11674,7 @@
         <v>47.327860000000001</v>
       </c>
       <c r="I123" s="11">
-        <v>71.262799999999999</v>
+        <v>71.26275634765625</v>
       </c>
       <c r="J123" s="11">
         <v>52.4</v>
@@ -11720,7 +11730,7 @@
         <v>100.4477</v>
       </c>
       <c r="I124" s="11">
-        <v>50.2121</v>
+        <v>50.212093353271484</v>
       </c>
       <c r="J124" s="11">
         <v>69.400000000000006</v>
@@ -11776,7 +11786,7 @@
         <v>69.167509999999993</v>
       </c>
       <c r="I125" s="11">
-        <v>72.654300000000006</v>
+        <v>72.654327392578125</v>
       </c>
       <c r="J125" s="11">
         <v>63.7</v>
@@ -11832,7 +11842,7 @@
         <v>28.433990000000001</v>
       </c>
       <c r="I126" s="11">
-        <v>35.189399999999999</v>
+        <v>35.189414978027344</v>
       </c>
       <c r="J126" s="11">
         <v>49.5</v>
@@ -11888,7 +11898,7 @@
         <v>45.653170000000003</v>
       </c>
       <c r="I127" s="11">
-        <v>27.7395</v>
+        <v>27.739459991455078</v>
       </c>
       <c r="J127" s="11">
         <v>74.5</v>
@@ -11944,7 +11954,7 @@
         <v>37.950650000000003</v>
       </c>
       <c r="I128" s="11">
-        <v>35.048000000000002</v>
+        <v>35.047966003417969</v>
       </c>
       <c r="J128" s="11">
         <v>59.8</v>
@@ -12000,7 +12010,7 @@
         <v>117.5663</v>
       </c>
       <c r="I129" s="11">
-        <v>47.826799999999999</v>
+        <v>47.826797485351562</v>
       </c>
       <c r="J129" s="11">
         <v>58.5</v>
@@ -12056,7 +12066,7 @@
         <v>186.62090000000001</v>
       </c>
       <c r="I130" s="11">
-        <v>58.0687</v>
+        <v>58.0687255859375</v>
       </c>
       <c r="J130" s="11">
         <v>80.5</v>
@@ -12112,7 +12122,7 @@
         <v>141.72020000000001</v>
       </c>
       <c r="I131" s="11">
-        <v>72.572100000000006</v>
+        <v>72.572135925292969</v>
       </c>
       <c r="J131" s="11">
         <v>38.700000000000003</v>
@@ -12168,7 +12178,7 @@
         <v>88.442459999999997</v>
       </c>
       <c r="I132" s="11">
-        <v>56.176099999999998</v>
+        <v>56.176078796386719</v>
       </c>
       <c r="J132" s="11">
         <v>77.599999999999994</v>
@@ -12224,7 +12234,7 @@
         <v>116.0401</v>
       </c>
       <c r="I133" s="11">
-        <v>61.8095</v>
+        <v>61.809478759765625</v>
       </c>
       <c r="J133" s="11">
         <v>65.2</v>
@@ -12280,7 +12290,7 @@
         <v>186.53909999999999</v>
       </c>
       <c r="I134" s="11">
-        <v>126.779</v>
+        <v>126.77857971191406</v>
       </c>
       <c r="J134" s="11">
         <v>103</v>
@@ -12336,7 +12346,7 @@
         <v>127.34869999999999</v>
       </c>
       <c r="I135" s="11">
-        <v>89.350399999999993</v>
+        <v>89.350440979003906</v>
       </c>
       <c r="J135" s="11">
         <v>99.8</v>
@@ -12392,7 +12402,7 @@
         <v>91.625209999999996</v>
       </c>
       <c r="I136" s="11">
-        <v>175.19200000000001</v>
+        <v>175.19227600097656</v>
       </c>
       <c r="J136" s="11">
         <v>99.1</v>
@@ -12448,7 +12458,7 @@
         <v>78.179479999999998</v>
       </c>
       <c r="I137" s="11">
-        <v>124.777</v>
+        <v>124.77665710449219</v>
       </c>
       <c r="J137" s="11">
         <v>72.400000000000006</v>
@@ -12504,7 +12514,7 @@
         <v>53.695779999999999</v>
       </c>
       <c r="I138" s="11">
-        <v>94.384399999999999</v>
+        <v>94.384407043457031</v>
       </c>
       <c r="J138" s="11">
         <v>67.7</v>
@@ -12560,7 +12570,7 @@
         <v>114.4254</v>
       </c>
       <c r="I139" s="11">
-        <v>162.874</v>
+        <v>162.87371826171875</v>
       </c>
       <c r="J139" s="11">
         <v>73.400000000000006</v>
@@ -12616,7 +12626,7 @@
         <v>85.725819999999999</v>
       </c>
       <c r="I140" s="11">
-        <v>193.61199999999999</v>
+        <v>193.61181640625</v>
       </c>
       <c r="J140" s="11">
         <v>61.4</v>
@@ -12672,7 +12682,7 @@
         <v>86.259249999999994</v>
       </c>
       <c r="I141" s="11">
-        <v>92.267499999999998</v>
+        <v>92.267471313476562</v>
       </c>
       <c r="J141" s="11">
         <v>58.9</v>
@@ -12728,7 +12738,7 @@
         <v>155.9118</v>
       </c>
       <c r="I142" s="11">
-        <v>124.11199999999999</v>
+        <v>124.11170196533203</v>
       </c>
       <c r="J142" s="11">
         <v>97.3</v>
@@ -12784,7 +12794,7 @@
         <v>256.0718</v>
       </c>
       <c r="I143" s="11">
-        <v>235.18600000000001</v>
+        <v>235.18559265136719</v>
       </c>
       <c r="J143" s="11">
         <v>133</v>
@@ -12840,7 +12850,7 @@
         <v>188.7567</v>
       </c>
       <c r="I144" s="11">
-        <v>146.62899999999999</v>
+        <v>146.629150390625</v>
       </c>
       <c r="J144" s="11">
         <v>86</v>
@@ -12896,7 +12906,7 @@
         <v>192.48840000000001</v>
       </c>
       <c r="I145" s="11">
-        <v>136.16</v>
+        <v>136.16011047363281</v>
       </c>
       <c r="J145" s="11">
         <v>74.7</v>
@@ -12952,7 +12962,7 @@
         <v>174.7227</v>
       </c>
       <c r="I146" s="11">
-        <v>105.815</v>
+        <v>105.81543731689453</v>
       </c>
       <c r="J146" s="11">
         <v>123</v>
@@ -13008,7 +13018,7 @@
         <v>121.99930000000001</v>
       </c>
       <c r="I147" s="11">
-        <v>135.76499999999999</v>
+        <v>135.76495361328125</v>
       </c>
       <c r="J147" s="11">
         <v>123</v>
@@ -13064,7 +13074,7 @@
         <v>144.3331</v>
       </c>
       <c r="I148" s="11">
-        <v>155.971</v>
+        <v>155.97053527832031</v>
       </c>
       <c r="J148" s="11">
         <v>123</v>
@@ -13120,7 +13130,7 @@
         <v>120.31100000000001</v>
       </c>
       <c r="I149" s="11">
-        <v>131.59100000000001</v>
+        <v>131.591064453125</v>
       </c>
       <c r="J149" s="11">
         <v>109</v>
@@ -13176,7 +13186,7 @@
         <v>112.80200000000001</v>
       </c>
       <c r="I150" s="11">
-        <v>114.316</v>
+        <v>114.31607818603516</v>
       </c>
       <c r="J150" s="11">
         <v>132</v>
@@ -13232,7 +13242,7 @@
         <v>136.32079999999999</v>
       </c>
       <c r="I151" s="11">
-        <v>98.400599999999997</v>
+        <v>98.400611877441406</v>
       </c>
       <c r="J151" s="11">
         <v>73.400000000000006</v>
@@ -13288,7 +13298,7 @@
         <v>79.354020000000006</v>
       </c>
       <c r="I152" s="11">
-        <v>141.06700000000001</v>
+        <v>141.06748962402344</v>
       </c>
       <c r="J152" s="11">
         <v>97.1</v>
@@ -13344,7 +13354,7 @@
         <v>122.8792</v>
       </c>
       <c r="I153" s="11">
-        <v>103.88</v>
+        <v>103.87956237792969</v>
       </c>
       <c r="J153" s="11">
         <v>57.7</v>
@@ -13400,7 +13410,7 @@
         <v>59.587850000000003</v>
       </c>
       <c r="I154" s="11">
-        <v>87.388800000000003</v>
+        <v>87.388771057128906</v>
       </c>
       <c r="J154" s="11">
         <v>117</v>
@@ -13456,7 +13466,7 @@
         <v>84.368049999999997</v>
       </c>
       <c r="I155" s="11">
-        <v>85.999099999999999</v>
+        <v>85.999076843261719</v>
       </c>
       <c r="J155" s="11">
         <v>88.2</v>
@@ -13512,7 +13522,7 @@
         <v>106.5706</v>
       </c>
       <c r="I156" s="11">
-        <v>68.559399999999997</v>
+        <v>68.559417724609375</v>
       </c>
       <c r="J156" s="11">
         <v>114</v>
@@ -13568,7 +13578,7 @@
         <v>76.332859999999997</v>
       </c>
       <c r="I157" s="11">
-        <v>78.486500000000007</v>
+        <v>78.486495971679688</v>
       </c>
       <c r="J157" s="11">
         <v>99.9</v>
@@ -13624,7 +13634,7 @@
         <v>105.5711</v>
       </c>
       <c r="I158" s="11">
-        <v>77.453900000000004</v>
+        <v>77.453849792480469</v>
       </c>
       <c r="J158" s="11">
         <v>105</v>
@@ -13680,7 +13690,7 @@
         <v>121.437</v>
       </c>
       <c r="I159" s="11">
-        <v>129.56899999999999</v>
+        <v>129.56900024414062</v>
       </c>
       <c r="J159" s="11">
         <v>106</v>
@@ -13736,7 +13746,7 @@
         <v>116.47020000000001</v>
       </c>
       <c r="I160" s="11">
-        <v>96.486900000000006</v>
+        <v>96.486854553222656</v>
       </c>
       <c r="J160" s="11">
         <v>98.6</v>
@@ -13792,7 +13802,7 @@
         <v>153.8355</v>
       </c>
       <c r="I161" s="11">
-        <v>94.168000000000006</v>
+        <v>94.168052673339844</v>
       </c>
       <c r="J161" s="11">
         <v>111</v>
@@ -13848,7 +13858,7 @@
         <v>156.381</v>
       </c>
       <c r="I162" s="11">
-        <v>113.86799999999999</v>
+        <v>113.86794281005859</v>
       </c>
       <c r="J162" s="11">
         <v>115</v>
@@ -13904,7 +13914,7 @@
         <v>143.11949999999999</v>
       </c>
       <c r="I163" s="11">
-        <v>151.37899999999999</v>
+        <v>151.37905883789062</v>
       </c>
       <c r="J163" s="11">
         <v>161</v>
@@ -13960,7 +13970,7 @@
         <v>193.8954</v>
       </c>
       <c r="I164" s="11">
-        <v>100.37</v>
+        <v>100.37033081054688</v>
       </c>
       <c r="J164" s="11">
         <v>144</v>
@@ -14016,7 +14026,7 @@
         <v>146.9263</v>
       </c>
       <c r="I165" s="11">
-        <v>89.108900000000006</v>
+        <v>89.108879089355469</v>
       </c>
       <c r="J165" s="11">
         <v>112</v>
@@ -14072,7 +14082,7 @@
         <v>111.5932</v>
       </c>
       <c r="I166" s="11">
-        <v>99.399500000000003</v>
+        <v>99.399482727050781</v>
       </c>
       <c r="J166" s="11">
         <v>126</v>
@@ -14128,7 +14138,7 @@
         <v>116.3798</v>
       </c>
       <c r="I167" s="11">
-        <v>88.999499999999998</v>
+        <v>88.999542236328125</v>
       </c>
       <c r="J167" s="11">
         <v>133</v>
@@ -14184,7 +14194,7 @@
         <v>137.21379999999999</v>
       </c>
       <c r="I168" s="11">
-        <v>107.062</v>
+        <v>107.06229400634766</v>
       </c>
       <c r="J168" s="11">
         <v>144</v>
@@ -14240,7 +14250,7 @@
         <v>179.4143</v>
       </c>
       <c r="I169" s="11">
-        <v>157.435</v>
+        <v>157.43473815917969</v>
       </c>
       <c r="J169" s="11">
         <v>110</v>
@@ -14296,7 +14306,7 @@
         <v>140.94579999999999</v>
       </c>
       <c r="I170" s="11">
-        <v>124.54900000000001</v>
+        <v>124.54881286621094</v>
       </c>
       <c r="J170" s="11">
         <v>87.9</v>
@@ -14352,7 +14362,7 @@
         <v>93.271109999999993</v>
       </c>
       <c r="I171" s="11">
-        <v>144.15199999999999</v>
+        <v>144.15167236328125</v>
       </c>
       <c r="J171" s="11">
         <v>103</v>
@@ -14408,7 +14418,7 @@
         <v>123.78570000000001</v>
       </c>
       <c r="I172" s="11">
-        <v>96.319199999999995</v>
+        <v>96.319206237792969</v>
       </c>
       <c r="J172" s="11">
         <v>99.3</v>
@@ -14464,7 +14474,7 @@
         <v>80.169269999999997</v>
       </c>
       <c r="I173" s="11">
-        <v>71.039900000000003</v>
+        <v>71.039939880371094</v>
       </c>
       <c r="J173" s="11">
         <v>104</v>
@@ -14520,7 +14530,7 @@
         <v>93.211039999999997</v>
       </c>
       <c r="I174" s="11">
-        <v>102.971</v>
+        <v>102.97064971923828</v>
       </c>
       <c r="J174" s="11">
         <v>138</v>
@@ -14576,7 +14586,7 @@
         <v>172.59469999999999</v>
       </c>
       <c r="I175" s="11">
-        <v>105.511</v>
+        <v>105.51095581054688</v>
       </c>
       <c r="J175" s="11">
         <v>97.7</v>
@@ -14632,7 +14642,7 @@
         <v>184.01230000000001</v>
       </c>
       <c r="I176" s="11">
-        <v>155.34</v>
+        <v>155.3404541015625</v>
       </c>
       <c r="J176" s="11">
         <v>126</v>
@@ -14688,7 +14698,7 @@
         <v>280.6148</v>
       </c>
       <c r="I177" s="11">
-        <v>272.87400000000002</v>
+        <v>272.87445068359375</v>
       </c>
       <c r="J177" s="11">
         <v>173</v>
@@ -14744,7 +14754,7 @@
         <v>377.84379999999999</v>
       </c>
       <c r="I178" s="11">
-        <v>186.78700000000001</v>
+        <v>186.78738403320312</v>
       </c>
       <c r="J178" s="11">
         <v>172</v>
@@ -14800,7 +14810,7 @@
         <v>217.8193</v>
       </c>
       <c r="I179" s="11">
-        <v>222.566</v>
+        <v>222.56591796875</v>
       </c>
       <c r="J179" s="11">
         <v>204</v>
@@ -14856,7 +14866,7 @@
         <v>327.94839999999999</v>
       </c>
       <c r="I180" s="11">
-        <v>224.14</v>
+        <v>224.14033508300781</v>
       </c>
       <c r="J180" s="11">
         <v>218</v>
@@ -14912,7 +14922,7 @@
         <v>203.20609999999999</v>
       </c>
       <c r="I181" s="11">
-        <v>249.339</v>
+        <v>249.33888244628906</v>
       </c>
       <c r="J181" s="11">
         <v>188</v>
@@ -14968,7 +14978,7 @@
         <v>193.76169999999999</v>
       </c>
       <c r="I182" s="11">
-        <v>183.11699999999999</v>
+        <v>183.11711120605469</v>
       </c>
       <c r="J182" s="11">
         <v>179</v>
@@ -15024,7 +15034,7 @@
         <v>127.25830000000001</v>
       </c>
       <c r="I183" s="11">
-        <v>180.22900000000001</v>
+        <v>180.22923278808594</v>
       </c>
       <c r="J183" s="11">
         <v>135</v>
@@ -15080,7 +15090,7 @@
         <v>112.18210000000001</v>
       </c>
       <c r="I184" s="11">
-        <v>239.41900000000001</v>
+        <v>239.41928100585938</v>
       </c>
       <c r="J184" s="11">
         <v>141</v>
@@ -15136,7 +15146,7 @@
         <v>139.8486</v>
       </c>
       <c r="I185" s="11">
-        <v>173.36799999999999</v>
+        <v>173.36813354492188</v>
       </c>
       <c r="J185" s="11">
         <v>190</v>
@@ -15192,7 +15202,7 @@
         <v>169.59649999999999</v>
       </c>
       <c r="I186" s="11">
-        <v>246.411</v>
+        <v>246.41078186035156</v>
       </c>
       <c r="J186" s="11">
         <v>148</v>
@@ -15248,7 +15258,7 @@
         <v>202.49010000000001</v>
       </c>
       <c r="I187" s="11">
-        <v>283.68900000000002</v>
+        <v>283.6890869140625</v>
       </c>
       <c r="J187" s="11">
         <v>141</v>
@@ -15304,7 +15314,7 @@
         <v>237.98159999999999</v>
       </c>
       <c r="I188" s="11">
-        <v>142.36500000000001</v>
+        <v>142.36514282226562</v>
       </c>
       <c r="J188" s="11">
         <v>126</v>
@@ -15360,7 +15370,7 @@
         <v>161.6062</v>
       </c>
       <c r="I189" s="11">
-        <v>166.005</v>
+        <v>166.00540161132812</v>
       </c>
       <c r="J189" s="11">
         <v>98.1</v>
@@ -15416,7 +15426,7 @@
         <v>227.42259999999999</v>
       </c>
       <c r="I190" s="11">
-        <v>152.36600000000001</v>
+        <v>152.36616516113281</v>
       </c>
       <c r="J190" s="11">
         <v>101</v>
@@ -15472,7 +15482,7 @@
         <v>174.70269999999999</v>
       </c>
       <c r="I191" s="11">
-        <v>163.22900000000001</v>
+        <v>163.22943115234375</v>
       </c>
       <c r="J191" s="11">
         <v>130</v>
@@ -15528,7 +15538,7 @@
         <v>214.81979999999999</v>
       </c>
       <c r="I192" s="11">
-        <v>141.81</v>
+        <v>141.81025695800781</v>
       </c>
       <c r="J192" s="11">
         <v>113</v>
@@ -15584,7 +15594,7 @@
         <v>170.51519999999999</v>
       </c>
       <c r="I193" s="11">
-        <v>153.565</v>
+        <v>153.56535339355469</v>
       </c>
       <c r="J193" s="11">
         <v>141</v>
@@ -15640,7 +15650,7 @@
         <v>198.88419999999999</v>
       </c>
       <c r="I194" s="11">
-        <v>133.149</v>
+        <v>133.14900207519531</v>
       </c>
       <c r="J194" s="11">
         <v>171</v>
@@ -15696,7 +15706,7 @@
         <v>152.42019999999999</v>
       </c>
       <c r="I195" s="11">
-        <v>138.351</v>
+        <v>138.35072326660156</v>
       </c>
       <c r="J195" s="11">
         <v>184</v>
@@ -15752,7 +15762,7 @@
         <v>201.00299999999999</v>
       </c>
       <c r="I196" s="11">
-        <v>155.18299999999999</v>
+        <v>155.18348693847656</v>
       </c>
       <c r="J196" s="11">
         <v>241</v>
@@ -15808,7 +15818,7 @@
         <v>131.46469999999999</v>
       </c>
       <c r="I197" s="11">
-        <v>148.751</v>
+        <v>148.75080871582031</v>
       </c>
       <c r="J197" s="11">
         <v>200</v>
@@ -15864,7 +15874,7 @@
         <v>65.217129999999997</v>
       </c>
       <c r="I198" s="11">
-        <v>122.285</v>
+        <v>122.28457641601562</v>
       </c>
       <c r="J198" s="11">
         <v>130</v>
@@ -15920,7 +15930,7 @@
         <v>126.3947</v>
       </c>
       <c r="I199" s="11">
-        <v>129.93799999999999</v>
+        <v>129.93832397460938</v>
       </c>
       <c r="J199" s="11">
         <v>135</v>
@@ -15976,7 +15986,7 @@
         <v>160.84450000000001</v>
       </c>
       <c r="I200" s="11">
-        <v>130.02600000000001</v>
+        <v>130.02572631835938</v>
       </c>
       <c r="J200" s="11">
         <v>172</v>
@@ -16032,7 +16042,7 @@
         <v>131.17689999999999</v>
       </c>
       <c r="I201" s="11">
-        <v>188.83</v>
+        <v>188.82957458496094</v>
       </c>
       <c r="J201" s="11">
         <v>126</v>
@@ -16088,7 +16098,7 @@
         <v>130.39099999999999</v>
       </c>
       <c r="I202" s="11">
-        <v>160.81800000000001</v>
+        <v>160.81842041015625</v>
       </c>
       <c r="J202" s="11">
         <v>170</v>
@@ -16144,7 +16154,7 @@
         <v>209.00710000000001</v>
       </c>
       <c r="I203" s="11">
-        <v>107.319</v>
+        <v>107.31888580322266</v>
       </c>
       <c r="J203" s="11">
         <v>153</v>
@@ -16200,7 +16210,7 @@
         <v>110.1592</v>
       </c>
       <c r="I204" s="11">
-        <v>79.370900000000006</v>
+        <v>79.370887756347656</v>
       </c>
       <c r="J204" s="11">
         <v>187</v>
@@ -16256,7 +16266,7 @@
         <v>166.10239999999999</v>
       </c>
       <c r="I205" s="11">
-        <v>103.19499999999999</v>
+        <v>103.19481658935547</v>
       </c>
       <c r="J205" s="11">
         <v>94.3</v>
@@ -16312,7 +16322,7 @@
         <v>106.1858</v>
       </c>
       <c r="I206" s="11">
-        <v>95.179900000000004</v>
+        <v>95.179939270019531</v>
       </c>
       <c r="J206" s="11">
         <v>116</v>
@@ -16368,7 +16378,7 @@
         <v>134.59870000000001</v>
       </c>
       <c r="I207" s="11">
-        <v>78.709900000000005</v>
+        <v>78.709884643554688</v>
       </c>
       <c r="J207" s="11">
         <v>136</v>
@@ -16424,7 +16434,7 @@
         <v>130.7784</v>
       </c>
       <c r="I208" s="11">
-        <v>66.1267</v>
+        <v>66.126670837402344</v>
       </c>
       <c r="J208" s="11">
         <v>129</v>
@@ -16480,7 +16490,7 @@
         <v>93.582229999999996</v>
       </c>
       <c r="I209" s="11">
-        <v>78.738900000000001</v>
+        <v>78.738861083984375</v>
       </c>
       <c r="J209" s="11">
         <v>103</v>
@@ -16536,7 +16546,7 @@
         <v>129.21799999999999</v>
       </c>
       <c r="I210" s="11">
-        <v>88.943899999999999</v>
+        <v>88.943901062011719</v>
       </c>
       <c r="J210" s="11">
         <v>105</v>
@@ -16592,7 +16602,7 @@
         <v>70.298320000000004</v>
       </c>
       <c r="I211" s="11">
-        <v>72.417299999999997</v>
+        <v>72.417304992675781</v>
       </c>
       <c r="J211" s="11">
         <v>105</v>
@@ -16648,7 +16658,7 @@
         <v>105.1964</v>
       </c>
       <c r="I212" s="11">
-        <v>104.407</v>
+        <v>104.40687561035156</v>
       </c>
       <c r="J212" s="11">
         <v>111</v>
@@ -16704,7 +16714,7 @@
         <v>142.96780000000001</v>
       </c>
       <c r="I213" s="11">
-        <v>133.45099999999999</v>
+        <v>133.45057678222656</v>
       </c>
       <c r="J213" s="11">
         <v>78.3</v>
@@ -16760,7 +16770,7 @@
         <v>177.005</v>
       </c>
       <c r="I214" s="11">
-        <v>115.322</v>
+        <v>115.32199859619141</v>
       </c>
       <c r="J214" s="11">
         <v>135</v>
@@ -16816,7 +16826,7 @@
         <v>150.62700000000001</v>
       </c>
       <c r="I215" s="11">
-        <v>91.5167</v>
+        <v>91.516685485839844</v>
       </c>
       <c r="J215" s="11">
         <v>104</v>
@@ -16872,7 +16882,7 @@
         <v>109.4573</v>
       </c>
       <c r="I216" s="11">
-        <v>119.68300000000001</v>
+        <v>119.68306732177734</v>
       </c>
       <c r="J216" s="11">
         <v>160</v>
@@ -16928,7 +16938,7 @@
         <v>152.4196</v>
       </c>
       <c r="I217" s="11">
-        <v>115.655</v>
+        <v>115.65457153320312</v>
       </c>
       <c r="J217" s="11">
         <v>120</v>
@@ -16984,7 +16994,7 @@
         <v>201.27250000000001</v>
       </c>
       <c r="I218" s="11">
-        <v>120.239</v>
+        <v>120.23883819580078</v>
       </c>
       <c r="J218" s="11">
         <v>99.3</v>
@@ -17040,7 +17050,7 @@
         <v>161.2988</v>
       </c>
       <c r="I219" s="11">
-        <v>98.449100000000001</v>
+        <v>98.449142456054688</v>
       </c>
       <c r="J219" s="11">
         <v>85.7</v>
@@ -17096,7 +17106,7 @@
         <v>80.55538</v>
       </c>
       <c r="I220" s="11">
-        <v>53.430399999999999</v>
+        <v>53.430370330810547</v>
       </c>
       <c r="J220" s="11">
         <v>109</v>
@@ -17152,7 +17162,7 @@
         <v>105.4915</v>
       </c>
       <c r="I221" s="11">
-        <v>52.308100000000003</v>
+        <v>52.308059692382812</v>
       </c>
       <c r="J221" s="11">
         <v>54.1</v>
@@ -17208,7 +17218,7 @@
         <v>113.3972</v>
       </c>
       <c r="I222" s="11">
-        <v>63.050699999999999</v>
+        <v>63.050682067871094</v>
       </c>
       <c r="J222" s="11">
         <v>146</v>
@@ -17264,7 +17274,7 @@
         <v>212.82470000000001</v>
       </c>
       <c r="I223" s="11">
-        <v>79.2637</v>
+        <v>79.263687133789062</v>
       </c>
       <c r="J223" s="11">
         <v>120</v>
@@ -17320,7 +17330,7 @@
         <v>176.398</v>
       </c>
       <c r="I224" s="11">
-        <v>50.592399999999998</v>
+        <v>50.592395782470703</v>
       </c>
       <c r="J224" s="11">
         <v>142</v>
@@ -17376,7 +17386,7 @@
         <v>158.68090000000001</v>
       </c>
       <c r="I225" s="11">
-        <v>77.5655</v>
+        <v>77.565513610839844</v>
       </c>
       <c r="J225" s="11">
         <v>114</v>
@@ -17432,7 +17442,7 @@
         <v>165.86699999999999</v>
       </c>
       <c r="I226" s="11">
-        <v>85.255200000000002</v>
+        <v>85.255157470703125</v>
       </c>
       <c r="J226" s="11">
         <v>125</v>
@@ -17488,7 +17498,7 @@
         <v>187.636</v>
       </c>
       <c r="I227" s="11">
-        <v>45.6004</v>
+        <v>45.600444793701172</v>
       </c>
       <c r="J227" s="11">
         <v>95.4</v>
@@ -17544,7 +17554,7 @@
         <v>193.55430000000001</v>
       </c>
       <c r="I228" s="11">
-        <v>47.6464</v>
+        <v>47.646373748779297</v>
       </c>
       <c r="J228" s="11">
         <v>96</v>
@@ -17600,7 +17610,7 @@
         <v>127.0861</v>
       </c>
       <c r="I229" s="11">
-        <v>77.321299999999994</v>
+        <v>77.321266174316406</v>
       </c>
       <c r="J229" s="11">
         <v>86.7</v>
@@ -17656,7 +17666,7 @@
         <v>203.9956</v>
       </c>
       <c r="I230" s="11">
-        <v>70.279600000000002</v>
+        <v>70.279624938964844</v>
       </c>
       <c r="J230" s="11">
         <v>97</v>
@@ -17712,7 +17722,7 @@
         <v>181.86089999999999</v>
       </c>
       <c r="I231" s="11">
-        <v>99.213399999999993</v>
+        <v>99.213386535644531</v>
       </c>
       <c r="J231" s="11">
         <v>119</v>
@@ -17768,7 +17778,7 @@
         <v>190.58179999999999</v>
       </c>
       <c r="I232" s="11">
-        <v>92.200900000000004</v>
+        <v>92.200859069824219</v>
       </c>
       <c r="J232" s="11">
         <v>104</v>
@@ -17824,7 +17834,7 @@
         <v>124.1682</v>
       </c>
       <c r="I233" s="11">
-        <v>47.387999999999998</v>
+        <v>47.388008117675781</v>
       </c>
       <c r="J233" s="11">
         <v>108</v>
@@ -17880,7 +17890,7 @@
         <v>131.46119999999999</v>
       </c>
       <c r="I234" s="11">
-        <v>53.013100000000001</v>
+        <v>53.013069152832031</v>
       </c>
       <c r="J234" s="11">
         <v>81.400000000000006</v>
@@ -17936,7 +17946,7 @@
         <v>454.00549999999998</v>
       </c>
       <c r="I235" s="11">
-        <v>144.26599999999999</v>
+        <v>144.26609802246094</v>
       </c>
       <c r="J235" s="11">
         <v>197</v>
@@ -17992,7 +18002,7 @@
         <v>331.66820000000001</v>
       </c>
       <c r="I236" s="11">
-        <v>78.066100000000006</v>
+        <v>78.066116333007812</v>
       </c>
       <c r="J236" s="11">
         <v>129</v>
@@ -18048,7 +18058,7 @@
         <v>223.12739999999999</v>
       </c>
       <c r="I237" s="11">
-        <v>41.014200000000002</v>
+        <v>41.014217376708984</v>
       </c>
       <c r="J237" s="11">
         <v>103</v>
@@ -18104,7 +18114,7 @@
         <v>219.07740000000001</v>
       </c>
       <c r="I238" s="11">
-        <v>32.883699999999997</v>
+        <v>32.883686065673828</v>
       </c>
       <c r="J238" s="11">
         <v>140</v>
@@ -18160,7 +18170,7 @@
         <v>148.26050000000001</v>
       </c>
       <c r="I239" s="11">
-        <v>38.686799999999998</v>
+        <v>38.686794281005859</v>
       </c>
       <c r="J239" s="11">
         <v>132</v>
@@ -18216,7 +18226,7 @@
         <v>322.22030000000001</v>
       </c>
       <c r="I240" s="11">
-        <v>72.805599999999998</v>
+        <v>72.805648803710938</v>
       </c>
       <c r="J240" s="11">
         <v>180</v>
@@ -18272,7 +18282,7 @@
         <v>246.8143</v>
       </c>
       <c r="I241" s="11">
-        <v>117.886</v>
+        <v>117.88623809814453</v>
       </c>
       <c r="J241" s="11">
         <v>159</v>
@@ -18328,7 +18338,7 @@
         <v>335.64150000000001</v>
       </c>
       <c r="I242" s="11">
-        <v>84.126599999999996</v>
+        <v>84.126556396484375</v>
       </c>
       <c r="J242" s="11">
         <v>113</v>
@@ -18384,7 +18394,7 @@
         <v>170.40049999999999</v>
       </c>
       <c r="I243" s="11">
-        <v>137.4</v>
+        <v>137.40043640136719</v>
       </c>
       <c r="J243" s="11">
         <v>114</v>
@@ -18440,7 +18450,7 @@
         <v>222.12299999999999</v>
       </c>
       <c r="I244" s="11">
-        <v>65.675200000000004</v>
+        <v>65.675193786621094</v>
       </c>
       <c r="J244" s="11">
         <v>98.6</v>
@@ -18496,7 +18506,7 @@
         <v>204.83879999999999</v>
       </c>
       <c r="I245" s="11">
-        <v>81.333799999999997</v>
+        <v>81.333839416503906</v>
       </c>
       <c r="J245" s="11">
         <v>61.9</v>
@@ -18552,7 +18562,7 @@
         <v>151.3844</v>
       </c>
       <c r="I246" s="11">
-        <v>39.263399999999997</v>
+        <v>39.26336669921875</v>
       </c>
       <c r="J246" s="11">
         <v>62.9</v>
@@ -18608,7 +18618,7 @@
         <v>192.2243</v>
       </c>
       <c r="I247" s="11">
-        <v>59.069899999999997</v>
+        <v>59.06988525390625</v>
       </c>
       <c r="J247" s="11">
         <v>99.6</v>
@@ -18664,7 +18674,7 @@
         <v>142.7124</v>
       </c>
       <c r="I248" s="11">
-        <v>62.029899999999998</v>
+        <v>62.029880523681641</v>
       </c>
       <c r="J248" s="11">
         <v>74</v>
@@ -18720,7 +18730,7 @@
         <v>104.7308</v>
       </c>
       <c r="I249" s="11">
-        <v>37.689500000000002</v>
+        <v>37.689472198486328</v>
       </c>
       <c r="J249" s="11">
         <v>31.7</v>
@@ -18776,7 +18786,7 @@
         <v>164.52680000000001</v>
       </c>
       <c r="I250" s="11">
-        <v>78.030600000000007</v>
+        <v>78.030647277832031</v>
       </c>
       <c r="J250" s="11">
         <v>91.2</v>
@@ -18832,7 +18842,7 @@
         <v>142.69749999999999</v>
       </c>
       <c r="I251" s="11">
-        <v>83.394800000000004</v>
+        <v>83.394752502441406</v>
       </c>
       <c r="J251" s="11">
         <v>66.3</v>
@@ -18888,7 +18898,7 @@
         <v>189.63560000000001</v>
       </c>
       <c r="I252" s="11">
-        <v>62.911999999999999</v>
+        <v>62.911979675292969</v>
       </c>
       <c r="J252" s="11">
         <v>63.3</v>
@@ -18944,7 +18954,7 @@
         <v>110.6977</v>
       </c>
       <c r="I253" s="11">
-        <v>81.988500000000002</v>
+        <v>81.988471984863281</v>
       </c>
       <c r="J253" s="11">
         <v>62.1</v>
@@ -19000,7 +19010,7 @@
         <v>150.03559999999999</v>
       </c>
       <c r="I254" s="11">
-        <v>39.425699999999999</v>
+        <v>39.425739288330078</v>
       </c>
       <c r="J254" s="11">
         <v>103</v>
@@ -19056,7 +19066,7 @@
         <v>97.528970000000001</v>
       </c>
       <c r="I255" s="11">
-        <v>79.909400000000005</v>
+        <v>79.909378051757812</v>
       </c>
       <c r="J255" s="11">
         <v>79.099999999999994</v>
@@ -19112,7 +19122,7 @@
         <v>113.2594</v>
       </c>
       <c r="I256" s="11">
-        <v>42.035400000000003</v>
+        <v>42.035430908203125</v>
       </c>
       <c r="J256" s="11">
         <v>77.5</v>
@@ -19168,7 +19178,7 @@
         <v>127.5361</v>
       </c>
       <c r="I257" s="11">
-        <v>34.923200000000001</v>
+        <v>34.923198699951172</v>
       </c>
       <c r="J257" s="11">
         <v>77.2</v>
@@ -19224,7 +19234,7 @@
         <v>178.8854</v>
       </c>
       <c r="I258" s="11">
-        <v>37.556800000000003</v>
+        <v>37.556758880615234</v>
       </c>
       <c r="J258" s="11">
         <v>135</v>
@@ -19280,7 +19290,7 @@
         <v>209.00210000000001</v>
       </c>
       <c r="I259" s="11">
-        <v>47.165700000000001</v>
+        <v>47.165748596191406</v>
       </c>
       <c r="J259" s="11">
         <v>129</v>
@@ -19336,7 +19346,7 @@
         <v>219.13720000000001</v>
       </c>
       <c r="I260" s="11">
-        <v>63.247199999999999</v>
+        <v>63.247226715087891</v>
       </c>
       <c r="J260" s="11">
         <v>101</v>
@@ -19392,7 +19402,7 @@
         <v>174.67609999999999</v>
       </c>
       <c r="I261" s="11">
-        <v>77.715100000000007</v>
+        <v>77.715065002441406</v>
       </c>
       <c r="J261" s="11">
         <v>87.7</v>
@@ -19448,7 +19458,7 @@
         <v>231.35669999999999</v>
       </c>
       <c r="I262" s="11">
-        <v>63.509500000000003</v>
+        <v>63.50946044921875</v>
       </c>
       <c r="J262" s="11">
         <v>109</v>
@@ -19504,7 +19514,7 @@
         <v>193.90710000000001</v>
       </c>
       <c r="I263" s="11">
-        <v>63.9161</v>
+        <v>63.916053771972656</v>
       </c>
       <c r="J263" s="11">
         <v>149</v>
@@ -19560,7 +19570,7 @@
         <v>148.1728</v>
       </c>
       <c r="I264" s="11">
-        <v>68.803200000000004</v>
+        <v>68.803184509277344</v>
       </c>
       <c r="J264" s="11">
         <v>139</v>
@@ -19616,7 +19626,7 @@
         <v>225.89789999999999</v>
       </c>
       <c r="I265" s="11">
-        <v>66.131699999999995</v>
+        <v>66.131683349609375</v>
       </c>
       <c r="J265" s="11">
         <v>188</v>
@@ -19672,7 +19682,7 @@
         <v>168.0872</v>
       </c>
       <c r="I266" s="11">
-        <v>64.738399999999999</v>
+        <v>64.738349914550781</v>
       </c>
       <c r="J266" s="11">
         <v>170</v>
@@ -19728,7 +19738,7 @@
         <v>155.94649999999999</v>
       </c>
       <c r="I267" s="11">
-        <v>50.119799999999998</v>
+        <v>50.119773864746094</v>
       </c>
       <c r="J267" s="11">
         <v>159</v>
@@ -19784,7 +19794,7 @@
         <v>248.37469999999999</v>
       </c>
       <c r="I268" s="11">
-        <v>40.585099999999997</v>
+        <v>40.585102081298828</v>
       </c>
       <c r="J268" s="11">
         <v>108</v>
@@ -19840,7 +19850,7 @@
         <v>198.25049999999999</v>
       </c>
       <c r="I269" s="11">
-        <v>60.453400000000002</v>
+        <v>60.453422546386719</v>
       </c>
       <c r="J269" s="11">
         <v>145</v>
@@ -19896,7 +19906,7 @@
         <v>145.92439999999999</v>
       </c>
       <c r="I270" s="11">
-        <v>83.642600000000002</v>
+        <v>83.642555236816406</v>
       </c>
       <c r="J270" s="11">
         <v>164</v>
@@ -19952,7 +19962,7 @@
         <v>171.3699</v>
       </c>
       <c r="I271" s="11">
-        <v>72.853399999999993</v>
+        <v>72.853439331054688</v>
       </c>
       <c r="J271" s="11">
         <v>115</v>
@@ -20008,7 +20018,7 @@
         <v>246.24189999999999</v>
       </c>
       <c r="I272" s="11">
-        <v>70.450800000000001</v>
+        <v>70.450836181640625</v>
       </c>
       <c r="J272" s="11">
         <v>88.9</v>
@@ -20064,7 +20074,7 @@
         <v>314.25810000000001</v>
       </c>
       <c r="I273" s="11">
-        <v>81.674800000000005</v>
+        <v>81.674781799316406</v>
       </c>
       <c r="J273" s="11">
         <v>113</v>
@@ -20120,7 +20130,7 @@
         <v>207.23429999999999</v>
       </c>
       <c r="I274" s="11">
-        <v>105.544</v>
+        <v>105.54432678222656</v>
       </c>
       <c r="J274" s="11">
         <v>112</v>
@@ -20176,7 +20186,7 @@
         <v>210.18510000000001</v>
       </c>
       <c r="I275" s="11">
-        <v>90.663899999999998</v>
+        <v>90.663871765136719</v>
       </c>
       <c r="J275" s="11">
         <v>95.3</v>
@@ -20232,7 +20242,7 @@
         <v>181.50479999999999</v>
       </c>
       <c r="I276" s="11">
-        <v>50.364699999999999</v>
+        <v>50.364681243896484</v>
       </c>
       <c r="J276" s="11">
         <v>89.5</v>
@@ -20288,7 +20298,7 @@
         <v>207.24610000000001</v>
       </c>
       <c r="I277" s="11">
-        <v>106.036</v>
+        <v>106.03553771972656</v>
       </c>
       <c r="J277" s="11">
         <v>150</v>
@@ -20344,7 +20354,7 @@
         <v>131.5076</v>
       </c>
       <c r="I278" s="11">
-        <v>48.135399999999997</v>
+        <v>48.135433197021484</v>
       </c>
       <c r="J278" s="11">
         <v>128</v>
@@ -20400,7 +20410,7 @@
         <v>304.09500000000003</v>
       </c>
       <c r="I279" s="11">
-        <v>92.649199999999993</v>
+        <v>92.649154663085938</v>
       </c>
       <c r="J279" s="11">
         <v>107</v>
@@ -20456,7 +20466,7 @@
         <v>498.05739999999997</v>
       </c>
       <c r="I280" s="11">
-        <v>110.098</v>
+        <v>110.09843444824219</v>
       </c>
       <c r="J280" s="11">
         <v>225</v>
@@ -20512,7 +20522,7 @@
         <v>374.94690000000003</v>
       </c>
       <c r="I281" s="11">
-        <v>160.822</v>
+        <v>160.82160949707031</v>
       </c>
       <c r="J281" s="11">
         <v>211</v>
@@ -20568,7 +20578,7 @@
         <v>397.71600000000001</v>
       </c>
       <c r="I282" s="11">
-        <v>167.75</v>
+        <v>167.75021362304688</v>
       </c>
       <c r="J282" s="11">
         <v>174</v>
@@ -20624,7 +20634,7 @@
         <v>278.87220000000002</v>
       </c>
       <c r="I283" s="11">
-        <v>75.147000000000006</v>
+        <v>75.14697265625</v>
       </c>
       <c r="J283" s="11">
         <v>156</v>
@@ -20680,7 +20690,7 @@
         <v>312.9316</v>
       </c>
       <c r="I284" s="11">
-        <v>107.754</v>
+        <v>107.75376129150391</v>
       </c>
       <c r="J284" s="11">
         <v>151</v>
@@ -20736,7 +20746,7 @@
         <v>215.73820000000001</v>
       </c>
       <c r="I285" s="11">
-        <v>115.057</v>
+        <v>115.05743408203125</v>
       </c>
       <c r="J285" s="11">
         <v>160</v>
@@ -20792,7 +20802,7 @@
         <v>295.31849999999997</v>
       </c>
       <c r="I286" s="11">
-        <v>82.274100000000004</v>
+        <v>82.274063110351562</v>
       </c>
       <c r="J286" s="11">
         <v>169</v>
@@ -20848,7 +20858,7 @@
         <v>443.74239999999998</v>
       </c>
       <c r="I287" s="11">
-        <v>95.4876</v>
+        <v>95.487632751464844</v>
       </c>
       <c r="J287" s="11">
         <v>174</v>
@@ -20904,7 +20914,7 @@
         <v>387.49450000000002</v>
       </c>
       <c r="I288" s="11">
-        <v>69.496700000000004</v>
+        <v>69.496719360351562</v>
       </c>
       <c r="J288" s="11">
         <v>279</v>
@@ -20960,7 +20970,7 @@
         <v>227.94399999999999</v>
       </c>
       <c r="I289" s="11">
-        <v>69.878500000000003</v>
+        <v>69.878494262695312</v>
       </c>
       <c r="J289" s="11">
         <v>142</v>
@@ -21016,7 +21026,7 @@
         <v>210.2321</v>
       </c>
       <c r="I290" s="11">
-        <v>83.661299999999997</v>
+        <v>83.661262512207031</v>
       </c>
       <c r="J290" s="11">
         <v>247</v>
@@ -21072,7 +21082,7 @@
         <v>223.45359999999999</v>
       </c>
       <c r="I291" s="11">
-        <v>51.7774</v>
+        <v>51.777389526367188</v>
       </c>
       <c r="J291" s="11">
         <v>137</v>
@@ -21128,7 +21138,7 @@
         <v>263.66320000000002</v>
       </c>
       <c r="I292" s="11">
-        <v>40.932299999999998</v>
+        <v>40.932342529296875</v>
       </c>
       <c r="J292" s="11">
         <v>175</v>
@@ -21184,7 +21194,7 @@
         <v>236.37899999999999</v>
       </c>
       <c r="I293" s="11">
-        <v>78.988299999999995</v>
+        <v>78.988319396972656</v>
       </c>
       <c r="J293" s="11">
         <v>134</v>
@@ -21240,7 +21250,7 @@
         <v>168.61250000000001</v>
       </c>
       <c r="I294" s="11">
-        <v>73.243799999999993</v>
+        <v>73.243804931640625</v>
       </c>
       <c r="J294" s="11">
         <v>59.5</v>
@@ -21296,7 +21306,7 @@
         <v>192.49770000000001</v>
       </c>
       <c r="I295" s="11">
-        <v>58.328499999999998</v>
+        <v>58.328456878662109</v>
       </c>
       <c r="J295" s="11">
         <v>105</v>
@@ -21352,7 +21362,7 @@
         <v>346.43419999999998</v>
       </c>
       <c r="I296" s="11">
-        <v>76.857200000000006</v>
+        <v>76.857254028320312</v>
       </c>
       <c r="J296" s="11">
         <v>61.5</v>
@@ -21408,7 +21418,7 @@
         <v>364.09980000000002</v>
       </c>
       <c r="I297" s="11">
-        <v>69.157600000000002</v>
+        <v>69.157646179199219</v>
       </c>
       <c r="J297" s="11">
         <v>41.3</v>
@@ -21464,7 +21474,7 @@
         <v>361.96710000000002</v>
       </c>
       <c r="I298" s="11">
-        <v>48.919600000000003</v>
+        <v>48.919631958007812</v>
       </c>
       <c r="J298" s="11">
         <v>103</v>
@@ -21520,7 +21530,7 @@
         <v>304.22579999999999</v>
       </c>
       <c r="I299" s="11">
-        <v>39.946300000000001</v>
+        <v>39.946323394775391</v>
       </c>
       <c r="J299" s="11">
         <v>70.7</v>
@@ -21576,7 +21586,7 @@
         <v>395.57159999999999</v>
       </c>
       <c r="I300" s="11">
-        <v>23.352799999999998</v>
+        <v>23.352756500244141</v>
       </c>
       <c r="J300" s="11">
         <v>103</v>
@@ -21632,7 +21642,7 @@
         <v>597.93619999999999</v>
       </c>
       <c r="I301" s="11">
-        <v>72.325299999999999</v>
+        <v>72.325332641601562</v>
       </c>
       <c r="J301" s="11">
         <v>128</v>
@@ -21688,7 +21698,7 @@
         <v>478.2045</v>
       </c>
       <c r="I302" s="11">
-        <v>70.024000000000001</v>
+        <v>70.023994445800781</v>
       </c>
       <c r="J302" s="11">
         <v>124</v>
@@ -21744,7 +21754,7 @@
         <v>394.1191</v>
       </c>
       <c r="I303" s="11">
-        <v>91.196600000000004</v>
+        <v>91.196632385253906</v>
       </c>
       <c r="J303" s="11">
         <v>120</v>
@@ -21800,7 +21810,7 @@
         <v>785.02560000000005</v>
       </c>
       <c r="I304" s="11">
-        <v>120.699</v>
+        <v>120.69873046875</v>
       </c>
       <c r="J304" s="11">
         <v>139</v>
@@ -21856,7 +21866,7 @@
         <v>707.87440000000004</v>
       </c>
       <c r="I305" s="11">
-        <v>90.130099999999999</v>
+        <v>90.130096435546875</v>
       </c>
       <c r="J305" s="11">
         <v>129</v>
@@ -21912,7 +21922,7 @@
         <v>616.04729999999995</v>
       </c>
       <c r="I306" s="11">
-        <v>69.116200000000006</v>
+        <v>69.116172790527344</v>
       </c>
       <c r="J306" s="11">
         <v>133</v>
@@ -21968,7 +21978,7 @@
         <v>589.16420000000005</v>
       </c>
       <c r="I307" s="11">
-        <v>65.4773</v>
+        <v>65.477294921875</v>
       </c>
       <c r="J307" s="11">
         <v>138</v>
@@ -22024,7 +22034,7 @@
         <v>765.0222</v>
       </c>
       <c r="I308" s="11">
-        <v>81.292100000000005</v>
+        <v>81.292091369628906</v>
       </c>
       <c r="J308" s="11">
         <v>125</v>
@@ -22080,7 +22090,7 @@
         <v>742.73869999999999</v>
       </c>
       <c r="I309" s="11">
-        <v>72.418099999999995</v>
+        <v>72.418113708496094</v>
       </c>
       <c r="J309" s="11">
         <v>117</v>
@@ -22136,7 +22146,7 @@
         <v>844.85469999999998</v>
       </c>
       <c r="I310" s="11">
-        <v>67.740200000000002</v>
+        <v>67.740234375</v>
       </c>
       <c r="J310" s="11">
         <v>173</v>
@@ -22192,7 +22202,7 @@
         <v>753.22969999999998</v>
       </c>
       <c r="I311" s="11">
-        <v>90.503</v>
+        <v>90.503028869628906</v>
       </c>
       <c r="J311" s="11">
         <v>96.8</v>
@@ -22248,7 +22258,7 @@
         <v>767.61749999999995</v>
       </c>
       <c r="I312" s="11">
-        <v>77.126300000000001</v>
+        <v>77.126251220703125</v>
       </c>
       <c r="J312" s="11">
         <v>86.2</v>
@@ -22304,7 +22314,7 @@
         <v>564.88620000000003</v>
       </c>
       <c r="I313" s="11">
-        <v>81.353200000000001</v>
+        <v>78.092086791992188</v>
       </c>
       <c r="J313" s="11">
         <v>78.599999999999994</v>
@@ -22330,6 +22340,369 @@
       </c>
       <c r="R313">
         <v>310.49697994126598</v>
+      </c>
+    </row>
+    <row r="314" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A314" t="s">
+        <v>79</v>
+      </c>
+      <c r="B314" s="15">
+        <v>1</v>
+      </c>
+      <c r="I314">
+        <v>50.974876403808594</v>
+      </c>
+    </row>
+    <row r="315" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A315" t="s">
+        <v>79</v>
+      </c>
+      <c r="B315" s="15">
+        <v>2</v>
+      </c>
+      <c r="I315">
+        <v>126.74948883056641</v>
+      </c>
+    </row>
+    <row r="316" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A316" t="s">
+        <v>79</v>
+      </c>
+      <c r="B316" s="15">
+        <v>3</v>
+      </c>
+      <c r="I316">
+        <v>72.3856201171875</v>
+      </c>
+    </row>
+    <row r="317" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A317" t="s">
+        <v>79</v>
+      </c>
+      <c r="B317" s="15">
+        <v>4</v>
+      </c>
+      <c r="I317">
+        <v>85.970741271972656</v>
+      </c>
+    </row>
+    <row r="318" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A318" t="s">
+        <v>79</v>
+      </c>
+      <c r="B318" s="15">
+        <v>5</v>
+      </c>
+      <c r="I318">
+        <v>48.450080871582031</v>
+      </c>
+    </row>
+    <row r="319" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A319" t="s">
+        <v>79</v>
+      </c>
+      <c r="B319" s="15">
+        <v>6</v>
+      </c>
+      <c r="I319">
+        <v>60.060012817382812</v>
+      </c>
+    </row>
+    <row r="320" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A320" t="s">
+        <v>79</v>
+      </c>
+      <c r="B320" s="15">
+        <v>7</v>
+      </c>
+      <c r="I320">
+        <v>55.642002105712891</v>
+      </c>
+    </row>
+    <row r="321" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A321" t="s">
+        <v>79</v>
+      </c>
+      <c r="B321" s="15">
+        <v>8</v>
+      </c>
+      <c r="I321">
+        <v>57.638164520263672</v>
+      </c>
+    </row>
+    <row r="322" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A322" t="s">
+        <v>79</v>
+      </c>
+      <c r="B322" s="15">
+        <v>9</v>
+      </c>
+      <c r="I322">
+        <v>32.909400939941406</v>
+      </c>
+    </row>
+    <row r="323" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A323" t="s">
+        <v>79</v>
+      </c>
+      <c r="B323" s="15">
+        <v>10</v>
+      </c>
+      <c r="I323">
+        <v>122.11404418945312</v>
+      </c>
+    </row>
+    <row r="324" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A324" t="s">
+        <v>79</v>
+      </c>
+      <c r="B324" s="15">
+        <v>11</v>
+      </c>
+      <c r="I324">
+        <v>104.73627471923828</v>
+      </c>
+    </row>
+    <row r="325" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A325" t="s">
+        <v>79</v>
+      </c>
+      <c r="B325" s="15">
+        <v>12</v>
+      </c>
+      <c r="I325">
+        <v>128.53721618652344</v>
+      </c>
+    </row>
+    <row r="326" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A326" t="s">
+        <v>80</v>
+      </c>
+      <c r="B326" s="15">
+        <v>1</v>
+      </c>
+      <c r="I326">
+        <v>129.90884399414062</v>
+      </c>
+    </row>
+    <row r="327" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A327" t="s">
+        <v>80</v>
+      </c>
+      <c r="B327" s="15">
+        <v>2</v>
+      </c>
+      <c r="I327">
+        <v>148.82550048828125</v>
+      </c>
+    </row>
+    <row r="328" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A328" t="s">
+        <v>80</v>
+      </c>
+      <c r="B328" s="15">
+        <v>3</v>
+      </c>
+      <c r="I328">
+        <v>91.722259521484375</v>
+      </c>
+    </row>
+    <row r="329" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A329" t="s">
+        <v>80</v>
+      </c>
+      <c r="B329" s="15">
+        <v>4</v>
+      </c>
+      <c r="I329">
+        <v>137.17509460449219</v>
+      </c>
+    </row>
+    <row r="330" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A330" t="s">
+        <v>80</v>
+      </c>
+      <c r="B330" s="15">
+        <v>5</v>
+      </c>
+      <c r="I330">
+        <v>83.037551879882812</v>
+      </c>
+    </row>
+    <row r="331" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A331" t="s">
+        <v>80</v>
+      </c>
+      <c r="B331" s="15">
+        <v>6</v>
+      </c>
+      <c r="I331">
+        <v>141.56019592285156</v>
+      </c>
+    </row>
+    <row r="332" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A332" t="s">
+        <v>80</v>
+      </c>
+      <c r="B332" s="15">
+        <v>7</v>
+      </c>
+      <c r="I332">
+        <v>193.13919067382812</v>
+      </c>
+    </row>
+    <row r="333" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A333" t="s">
+        <v>80</v>
+      </c>
+      <c r="B333" s="15">
+        <v>8</v>
+      </c>
+      <c r="I333">
+        <v>117.74303436279297</v>
+      </c>
+    </row>
+    <row r="334" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A334" t="s">
+        <v>80</v>
+      </c>
+      <c r="B334" s="15">
+        <v>9</v>
+      </c>
+      <c r="I334">
+        <v>143.18696594238281</v>
+      </c>
+    </row>
+    <row r="335" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A335" t="s">
+        <v>80</v>
+      </c>
+      <c r="B335" s="15">
+        <v>10</v>
+      </c>
+      <c r="I335">
+        <v>152.86872863769531</v>
+      </c>
+    </row>
+    <row r="336" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A336" t="s">
+        <v>80</v>
+      </c>
+      <c r="B336" s="15">
+        <v>11</v>
+      </c>
+      <c r="I336">
+        <v>105.32082366943359</v>
+      </c>
+    </row>
+    <row r="337" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A337" t="s">
+        <v>80</v>
+      </c>
+      <c r="B337" s="15">
+        <v>12</v>
+      </c>
+      <c r="I337">
+        <v>142.25140380859375</v>
+      </c>
+    </row>
+    <row r="338" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A338" t="s">
+        <v>81</v>
+      </c>
+      <c r="B338" s="15">
+        <v>1</v>
+      </c>
+      <c r="I338">
+        <v>169.27558898925781</v>
+      </c>
+    </row>
+    <row r="339" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A339" t="s">
+        <v>81</v>
+      </c>
+      <c r="B339" s="15">
+        <v>2</v>
+      </c>
+      <c r="I339">
+        <v>176.33804321289062</v>
+      </c>
+    </row>
+    <row r="340" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A340" t="s">
+        <v>81</v>
+      </c>
+      <c r="B340" s="15">
+        <v>3</v>
+      </c>
+      <c r="I340">
+        <v>132.86566162109375</v>
+      </c>
+    </row>
+    <row r="341" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A341" t="s">
+        <v>81</v>
+      </c>
+      <c r="B341" s="15">
+        <v>4</v>
+      </c>
+      <c r="I341">
+        <v>157.31352233886719</v>
+      </c>
+    </row>
+    <row r="342" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A342" t="s">
+        <v>81</v>
+      </c>
+      <c r="B342" s="15">
+        <v>5</v>
+      </c>
+      <c r="I342">
+        <v>98.961532592773438</v>
+      </c>
+    </row>
+    <row r="343" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A343" t="s">
+        <v>81</v>
+      </c>
+      <c r="B343" s="15">
+        <v>6</v>
+      </c>
+      <c r="I343">
+        <v>145.55709838867188</v>
+      </c>
+    </row>
+    <row r="344" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A344" t="s">
+        <v>81</v>
+      </c>
+      <c r="B344" s="15">
+        <v>7</v>
+      </c>
+      <c r="I344">
+        <v>81.778083801269531</v>
+      </c>
+    </row>
+    <row r="345" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A345" t="s">
+        <v>81</v>
+      </c>
+      <c r="B345" s="15">
+        <v>8</v>
+      </c>
+      <c r="I345">
+        <v>122.74759674072266</v>
+      </c>
+    </row>
+    <row r="346" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A346" t="s">
+        <v>81</v>
+      </c>
+      <c r="B346" s="15">
+        <v>9</v>
+      </c>
+      <c r="I346">
+        <v>168.50311279296875</v>
       </c>
     </row>
   </sheetData>
@@ -22349,6 +22722,9 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A314:B346" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 

</xml_diff>